<commit_message>
ci(dev): publish dev build from 0f13a3f4243ee74d0b61e5e75c725338e0588c38 0f13a3f4243ee74d0b61e5e75c725338e0588c38
</commit_message>
<xml_diff>
--- a/dev/CodeSystem-PSCED.xlsx
+++ b/dev/CodeSystem-PSCED.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
+    <sheet name="Concepts" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="52">
   <si>
     <t>Property</t>
   </si>
@@ -23,13 +24,13 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://doh.gov.ph/fhir/ph-core/CodeSystem/PSCED</t>
+    <t>https://psa.gov.ph/classification/psced/level</t>
   </si>
   <si>
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -59,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-08T04:20:57+00:00</t>
+    <t>2026-04-10T05:32:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -110,13 +111,64 @@
     <t>Content</t>
   </si>
   <si>
-    <t>not-present</t>
+    <t>example</t>
   </si>
   <si>
     <t>Supplements</t>
   </si>
   <si>
     <t>Count</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>C201301</t>
+  </si>
+  <si>
+    <t>Elementary Graduate</t>
+  </si>
+  <si>
+    <t>Completed elementary education</t>
+  </si>
+  <si>
+    <t>C201302</t>
+  </si>
+  <si>
+    <t>High School Graduate</t>
+  </si>
+  <si>
+    <t>Completed secondary education</t>
+  </si>
+  <si>
+    <t>C201303</t>
+  </si>
+  <si>
+    <t>College Graduate</t>
+  </si>
+  <si>
+    <t>Completed bachelor's degree</t>
+  </si>
+  <si>
+    <t>C201304</t>
+  </si>
+  <si>
+    <t>Postgraduate</t>
+  </si>
+  <si>
+    <t>Completed master's or doctoral degree</t>
   </si>
 </sst>
 </file>
@@ -420,4 +472,84 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s" s="2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s" s="2">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s" s="2">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>